<commit_message>
fix: clarify container booking fields
</commit_message>
<xml_diff>
--- a/public/templates/NXP-038_Container_Import_Cong_Ty_Van_Chuyen.xlsx
+++ b/public/templates/NXP-038_Container_Import_Cong_Ty_Van_Chuyen.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CongTyVanChuyen" sheetId="1" r:id="R0baa8fe578574305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="Rad7e2487daa24f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CongTyVanChuyen" sheetId="1" r:id="R36a9df9b80314382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="R594c86ac008d4562"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -531,7 +531,7 @@
         <x:v>gross_weight_kg</x:v>
       </x:c>
       <x:c r="I1" s="8" t="str">
-        <x:v>requested_pickup_date</x:v>
+        <x:v>requested_service_date</x:v>
       </x:c>
       <x:c r="J1" s="8" t="str">
         <x:v>bl_booking_number</x:v>
@@ -680,7 +680,9 @@
       <x:c r="H5" s="23" t="n">
         <x:v>26000</x:v>
       </x:c>
-      <x:c r="I5" s="26"/>
+      <x:c r="I5" s="26" t="n">
+        <x:v>46113</x:v>
+      </x:c>
       <x:c r="J5" s="19" t="str">
         <x:v>DADG02202800</x:v>
       </x:c>
@@ -752,7 +754,9 @@
       <x:c r="H7" s="23" t="n">
         <x:v>32500</x:v>
       </x:c>
-      <x:c r="I7" s="26"/>
+      <x:c r="I7" s="26" t="n">
+        <x:v>46083</x:v>
+      </x:c>
       <x:c r="J7" s="19" t="str">
         <x:v>DADG02482400</x:v>
       </x:c>
@@ -824,7 +828,9 @@
       <x:c r="H9" s="23" t="n">
         <x:v>9496</x:v>
       </x:c>
-      <x:c r="I9" s="26"/>
+      <x:c r="I9" s="26" t="n">
+        <x:v>46113</x:v>
+      </x:c>
       <x:c r="J9" s="19" t="str">
         <x:v>DADG02410900</x:v>
       </x:c>
@@ -896,7 +902,9 @@
       <x:c r="H11" s="23" t="n">
         <x:v>32500</x:v>
       </x:c>
-      <x:c r="I11" s="26"/>
+      <x:c r="I11" s="26" t="n">
+        <x:v>46083</x:v>
+      </x:c>
       <x:c r="J11" s="19" t="str">
         <x:v>DADG02482400</x:v>
       </x:c>
@@ -12828,7 +12836,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90cfc43987944186"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10df6e1f53cf4c02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12894,7 +12902,7 @@
         <x:v>Trường bắt buộc</x:v>
       </x:c>
       <x:c r="B6" s="42" t="str">
-        <x:v>container_number, container_type, movement_type, transport_company_name; pickup_request cần requested_pickup_date</x:v>
+        <x:v>container_number, container_type, movement_type, requested_service_date, transport_company_name.</x:v>
       </x:c>
       <x:c r="C6" s="39"/>
       <x:c r="D6" s="39"/>
@@ -12918,7 +12926,7 @@
         <x:v>Lưu ý</x:v>
       </x:c>
       <x:c r="B8" s="42" t="str">
-        <x:v>Dữ liệu được lưu ở trạng thái chờ đối soát với nguồn cảng. Chỉ khai báo nhu cầu nhận hoặc đưa Container vào cảng.</x:v>
+        <x:v>requested_service_date là ngày mong muốn nhận hoặc đưa Container vào cảng, dùng định dạng YYYY-MM-DD.</x:v>
       </x:c>
       <x:c r="C8" s="39"/>
       <x:c r="D8" s="39"/>

</xml_diff>

<commit_message>
fix: simplify container declarations
</commit_message>
<xml_diff>
--- a/public/templates/NXP-038_Container_Import_Cong_Ty_Van_Chuyen.xlsx
+++ b/public/templates/NXP-038_Container_Import_Cong_Ty_Van_Chuyen.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CongTyVanChuyen" sheetId="1" r:id="R36a9df9b80314382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="R594c86ac008d4562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CongTyVanChuyen" sheetId="1" r:id="R64bbc1ac55b049ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="Rb965c9538e0f4b1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12836,7 +12836,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10df6e1f53cf4c02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R853cb10df58f4758"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12911,10 +12911,10 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="41" t="str">
-        <x:v>Trạng thái dữ liệu</x:v>
+        <x:v>Mục đích dữ liệu</x:v>
       </x:c>
       <x:c r="B7" s="42" t="str">
-        <x:v>pending_verification</x:v>
+        <x:v>Dữ liệu đầu vào tạo Booking</x:v>
       </x:c>
       <x:c r="C7" s="39"/>
       <x:c r="D7" s="39"/>

</xml_diff>